<commit_message>
Agregado producto: TEG HEUER F1
</commit_message>
<xml_diff>
--- a/Descripcion.xlsx
+++ b/Descripcion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -658,6 +658,26 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>teg_heuer_f1_1789586665.jpeg</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TEG HEUER F1</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Reloj Tag Heuer F1 yellow</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregado producto: Tag Heuer
</commit_message>
<xml_diff>
--- a/Descripcion.xlsx
+++ b/Descripcion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -641,60 +641,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tag_heuer_f1_1789586555.jpeg</t>
+          <t>tag_heuer_1789587051.jpeg</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TAG HEUER F1</t>
+          <t>Tag Heuer</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>300000</v>
+        <v>100000</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>F1 amarillo</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>teg_heuer_f1_1789586665.jpeg</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>TEG HEUER F1</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Reloj Tag Heuer F1 yellow</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>teg_heuer_f1_1789586811.jpeg</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>TEG HEUER F1</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Reloj Tag Heuer F1 yellow</t>
+          <t>Reloj tag F1 amarillo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregado producto: Reloj TAG
</commit_message>
<xml_diff>
--- a/Descripcion.xlsx
+++ b/Descripcion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -658,6 +658,26 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>reloj_tag_1789589110.jpeg</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Reloj TAG</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TAG F1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>